<commit_message>
Update FX rates: 2026-04-13T08:30:10Z
</commit_message>
<xml_diff>
--- a/banks/fx_rates.xlsx
+++ b/banks/fx_rates.xlsx
@@ -449,7 +449,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -464,19 +464,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>24.42</t>
+          <t>24.60</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>25.99</t>
+          <t>26.19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -491,19 +491,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>63.06</t>
+          <t>63.17</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>67.85</t>
+          <t>68.03</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -518,19 +518,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>65.03</t>
+          <t>65.32</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>68.92</t>
+          <t>69.24</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -545,19 +545,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>114.09</t>
+          <t>114.68</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>120.19</t>
+          <t>120.84</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -584,7 +584,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -599,19 +599,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>13.99</t>
+          <t>14.08</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>14.99</t>
+          <t>15.09</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -626,19 +626,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>105.95</t>
+          <t>106.65</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>110.61</t>
+          <t>111.36</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -653,19 +653,19 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>120.87</t>
+          <t>121.51</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>127.71</t>
+          <t>128.47</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -680,19 +680,19 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.45</t>
+          <t>11.54</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>12.18</t>
+          <t>12.28</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -707,19 +707,19 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.5588</t>
+          <t>0.5608</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.6046</t>
+          <t>0.6070</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -734,19 +734,19 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.0596</t>
+          <t>0.0597</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.0655</t>
+          <t>0.0656</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -773,7 +773,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -788,19 +788,19 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.27</t>
+          <t>9.31</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>10.23</t>
+          <t>10.26</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -815,19 +815,19 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>51.87</t>
+          <t>52.00</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>56.45</t>
+          <t>56.58</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -842,19 +842,19 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>232.70</t>
+          <t>234.40</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>248.23</t>
+          <t>250.12</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -869,19 +869,19 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>23.90</t>
+          <t>24.08</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>25.44</t>
+          <t>25.63</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -896,19 +896,19 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>9.49</t>
+          <t>9.51</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>10.44</t>
+          <t>10.47</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -923,19 +923,19 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>71.35</t>
+          <t>71.71</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>74.00</t>
+          <t>74.45</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -950,19 +950,19 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2.77</t>
+          <t>2.78</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2.98</t>
+          <t>3.00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -977,19 +977,19 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>90.92</t>
+          <t>91.58</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>94.24</t>
+          <t>94.96</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1009,14 +1009,14 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>5.89</t>
+          <t>5.88</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1043,7 +1043,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1070,7 +1070,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1085,19 +1085,19 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>237.67</t>
+          <t>239.53</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>253.15</t>
+          <t>255.08</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1112,19 +1112,19 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>292.38</t>
+          <t>294.61</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>311.73</t>
+          <t>314.21</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1139,19 +1139,19 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>24.51</t>
+          <t>24.70</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>26.27</t>
+          <t>26.47</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1178,7 +1178,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1193,12 +1193,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>12.94</t>
+          <t>13.03</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>14.17</t>
+          <t>14.27</t>
         </is>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1261,19 +1261,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>92.4</t>
+          <t>92.9</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>93.25</t>
+          <t>93.75</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1288,19 +1288,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>24.66</t>
+          <t>24.79</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>25.92</t>
+          <t>26.04</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1315,19 +1315,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>64.46</t>
+          <t>64.51</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>66.73</t>
+          <t>66.79</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1354,7 +1354,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1369,19 +1369,19 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>238.52</t>
+          <t>239.77</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>253.97</t>
+          <t>255.27</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1396,19 +1396,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>66.33</t>
+          <t>66.53</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>67.93</t>
+          <t>68.12</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1423,19 +1423,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>115.4</t>
+          <t>115.82</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>119.47</t>
+          <t>119.89</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1462,7 +1462,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1477,19 +1477,19 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>14.39</t>
+          <t>14.47</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>14.64</t>
+          <t>14.72</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1504,19 +1504,19 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>107.16</t>
+          <t>107.73</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>109.83</t>
+          <t>110.41</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1531,19 +1531,19 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>123.12</t>
+          <t>123.65</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>125.93</t>
+          <t>126.48</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1558,19 +1558,19 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.75</t>
+          <t>11.82</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11.94</t>
+          <t>12.01</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1597,7 +1597,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1612,19 +1612,19 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>57.65</t>
+          <t>57.8</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>58.92</t>
+          <t>59.06</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1651,7 +1651,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1678,7 +1678,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1693,19 +1693,19 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>292.77</t>
+          <t>294.57</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>308.52</t>
+          <t>310.4</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1732,7 +1732,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1759,7 +1759,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1774,19 +1774,19 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>9.72</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>9.85</t>
+          <t>9.88</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1801,19 +1801,19 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>53.17</t>
+          <t>53.23</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>55.34</t>
+          <t>55.41</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1828,19 +1828,19 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>234.81</t>
+          <t>235.89</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>248.3</t>
+          <t>249.42</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1867,7 +1867,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1882,19 +1882,19 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>24.84</t>
+          <t>24.97</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>26.1</t>
+          <t>26.25</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1921,7 +1921,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1936,19 +1936,19 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>24.23</t>
+          <t>24.01</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>25.38</t>
+          <t>25.96</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1968,14 +1968,14 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>10.06</t>
+          <t>10.08</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1990,19 +1990,19 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>71.92</t>
+          <t>72.22</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>73.74</t>
+          <t>74.04</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2022,14 +2022,14 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>296</t>
+          <t>297</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2056,7 +2056,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2071,12 +2071,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>5.51</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>5.79</t>
+          <t>5.78</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2124,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2139,19 +2139,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>90.8</t>
+          <t>91.63</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>93.84</t>
+          <t>94.69</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2166,19 +2166,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>105.58</t>
+          <t>106.48</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>110.4</t>
+          <t>111.33</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2193,19 +2193,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>120.96</t>
+          <t>121.84</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>127.35</t>
+          <t>128.27</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2220,19 +2220,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>63.79</t>
+          <t>64.05</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>67.65</t>
+          <t>67.92</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2247,19 +2247,19 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>65.11</t>
+          <t>65.52</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>68.72</t>
+          <t>69.16</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2274,19 +2274,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>71.23</t>
+          <t>71.77</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>73.89</t>
+          <t>74.44</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2301,19 +2301,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>56.51</t>
+          <t>56.8</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>59.85</t>
+          <t>60.16</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2328,19 +2328,19 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>24.38</t>
+          <t>24.6</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>25.95</t>
+          <t>26.19</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2355,19 +2355,19 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>114.16</t>
+          <t>114.96</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>119.79</t>
+          <t>120.62</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2382,19 +2382,19 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>23.88</t>
+          <t>24.1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>25.39</t>
+          <t>25.62</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2409,19 +2409,19 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>24.58</t>
+          <t>24.81</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>26.32</t>
+          <t>26.56</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2436,19 +2436,19 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.6</t>
+          <t>9.64</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>10.35</t>
+          <t>10.39</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2463,19 +2463,19 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13.94</t>
+          <t>14.06</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14.95</t>
+          <t>15.07</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2490,19 +2490,19 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.37</t>
+          <t>9.42</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10.13</t>
+          <t>10.18</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2517,19 +2517,19 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>52.79</t>
+          <t>53.01</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>55.71</t>
+          <t>55.94</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2544,19 +2544,19 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>11.45</t>
+          <t>11.56</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>12.14</t>
+          <t>12.26</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2571,19 +2571,19 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>287.85</t>
+          <t>290.58</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>313.82</t>
+          <t>316.77</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2598,19 +2598,19 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.78</t>
+          <t>2.79</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.96</t>
+          <t>2.98</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2637,7 +2637,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2652,19 +2652,19 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>233.19</t>
+          <t>235.33</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>247.48</t>
+          <t>249.72</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2679,19 +2679,19 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.0596</t>
+          <t>0.0598</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0.0653</t>
+          <t>0.0655</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2706,19 +2706,19 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>12.92</t>
+          <t>13.04</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>14.15</t>
+          <t>14.27</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2733,19 +2733,19 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>24.49</t>
+          <t>24.64</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>26.31</t>
+          <t>26.49</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2760,19 +2760,19 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>237.21</t>
+          <t>239.51</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>252.84</t>
+          <t>255.14</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2787,12 +2787,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>22.22</t>
+          <t>22.4</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>24.36</t>
+          <t>24.55</t>
         </is>
       </c>
     </row>
@@ -2855,12 +2855,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>92.19</t>
+          <t>93.13</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>92.75</t>
+          <t>93.69</t>
         </is>
       </c>
     </row>
@@ -2882,12 +2882,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>72.18</t>
+          <t>72.80</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>72.97</t>
+          <t>73.60</t>
         </is>
       </c>
     </row>
@@ -2909,12 +2909,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.88</t>
+          <t>9.95</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9.99</t>
+          <t>10.06</t>
         </is>
       </c>
     </row>
@@ -2936,12 +2936,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>53.73</t>
+          <t>54.09</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>54.32</t>
+          <t>54.68</t>
         </is>
       </c>
     </row>
@@ -2963,12 +2963,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9.69</t>
+          <t>9.73</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>9.79</t>
+          <t>9.84</t>
         </is>
       </c>
     </row>
@@ -2990,12 +2990,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>29.08</t>
+          <t>29.37</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>29.52</t>
+          <t>29.81</t>
         </is>
       </c>
     </row>
@@ -3017,12 +3017,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>57.75</t>
+          <t>58.12</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>58.39</t>
+          <t>58.77</t>
         </is>
       </c>
     </row>
@@ -3044,12 +3044,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>11.73</t>
+          <t>11.86</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>11.86</t>
+          <t>11.99</t>
         </is>
       </c>
     </row>
@@ -3071,12 +3071,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>123.52</t>
+          <t>124.59</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>124.76</t>
+          <t>125.84</t>
         </is>
       </c>
     </row>
@@ -3098,12 +3098,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>107.60</t>
+          <t>108.61</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>108.69</t>
+          <t>109.70</t>
         </is>
       </c>
     </row>
@@ -3125,12 +3125,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>14.38</t>
+          <t>14.51</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>14.54</t>
+          <t>14.67</t>
         </is>
       </c>
     </row>
@@ -3152,12 +3152,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>116.28</t>
+          <t>117.31</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>117.56</t>
+          <t>118.61</t>
         </is>
       </c>
     </row>
@@ -3179,12 +3179,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>66.49</t>
+          <t>67.02</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>67.22</t>
+          <t>67.76</t>
         </is>
       </c>
     </row>
@@ -3206,12 +3206,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>64.94</t>
+          <t>65.32</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>65.66</t>
+          <t>66.04</t>
         </is>
       </c>
     </row>
@@ -3233,12 +3233,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>24.98</t>
+          <t>25.23</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>25.35</t>
+          <t>25.61</t>
         </is>
       </c>
     </row>

</xml_diff>